<commit_message>
Recaudación inicia F3 (5-jul, flexible) + modelo en hold + registro de trazabilidad
- estado.json: inicio_recaudacion (F3/5-jul, pago lump o por cuotas), profondo1_fechas
  (31-jul→2-ago), asignacion_entradas (pendiente, se revisa después).
- build_flujo.py: cuotas desde julio (no junio); el flujo revela que junio-julio quedan
  en negativo (F1/F2 se frontean) hasta que entran rifa+cuotas en agosto. Modelo EN HOLD.
- build_trazabilidad.py → preparacion/TRAZABILIDAD.md: registro generado desde estado.json
  con cada hecho, su estado y su fuente (trazabilidad de contenido y de fuentes).
- TODO PASS.

https://claude.ai/code/session_016scja59CycFFrqKgYsUPWh
</commit_message>
<xml_diff>
--- a/Flujo_Caja_ETC88.xlsx
+++ b/Flujo_Caja_ETC88.xlsx
@@ -143,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -195,6 +195,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -1131,14 +1134,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>FLUJO DE CAJA MENSUAL · arranca en –$23,600 (deuda) · [ESCENARIO] de fechas</t>
+          <t>FLUJO DE CAJA MENSUAL · arranca en –$23,600 · recaudación inicia F3 (5-jul) · [EN HOLD]</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Objetivo: que el SALDO no se vuelva crítico antes de un pago grande (casa, transporte). Las fechas son supuestos a confirmar.</t>
+          <t>Recaudación de cuotas inicia en la 1ra formación de julio (pago lump o por cuotas, a decisión del miembro). Profondo #1: 31-jul→2-ago. JUNIO sin ingresos: F1/F2 se frontean. Fechas [ESCENARIO] a confirmar.</t>
         </is>
       </c>
     </row>
@@ -1184,11 +1187,11 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Cuotas equipo ($500/mes) [PROPUESTA]</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="n">
-        <v>23500</v>
+          <t>Cuotas equipo ($500/mes desde F3, flexible) [PROPUESTA]</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="n">
+        <v>0</v>
       </c>
       <c r="C6" s="7" t="n">
         <v>23500</v>
@@ -1200,13 +1203,13 @@
         <v>23500</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>94000</v>
+        <v>70500</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Cuotas participantes [ESTIMADO]</t>
+          <t>Cuotas participantes (desde jul) [ESTIMADO]</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
@@ -1228,7 +1231,7 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Rifa neta (Profondo #1) [ESCENARIO]</t>
+          <t>Rifa neta (Profondo #1, 31-jul→2-ago) [ESCENARIO]</t>
         </is>
       </c>
       <c r="B8" s="18" t="n">
@@ -1285,10 +1288,10 @@
         <v>40000</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>25566</v>
+        <v>49066</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>90566</v>
+        <v>114066</v>
       </c>
     </row>
     <row r="11">
@@ -1298,23 +1301,23 @@
         </is>
       </c>
       <c r="B11" s="20" t="n">
-        <v>23500</v>
-      </c>
-      <c r="C11" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="21" t="n">
         <v>96200</v>
       </c>
-      <c r="D11" s="20" t="n">
+      <c r="D11" s="21" t="n">
         <v>354800</v>
       </c>
-      <c r="E11" s="20" t="n">
-        <v>109066</v>
-      </c>
-      <c r="F11" s="20" t="n">
+      <c r="E11" s="21" t="n">
+        <v>132566</v>
+      </c>
+      <c r="F11" s="21" t="n">
         <v>583566</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>SALIDAS</t>
         </is>
@@ -1541,24 +1544,24 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="22" t="inlineStr">
+      <c r="A24" s="23" t="inlineStr">
         <is>
           <t>TOTAL SALIDAS</t>
         </is>
       </c>
-      <c r="B24" s="23" t="n">
+      <c r="B24" s="24" t="n">
         <v>5300</v>
       </c>
-      <c r="C24" s="23" t="n">
+      <c r="C24" s="24" t="n">
         <v>75300</v>
       </c>
-      <c r="D24" s="23" t="n">
+      <c r="D24" s="24" t="n">
         <v>206400</v>
       </c>
-      <c r="E24" s="23" t="n">
+      <c r="E24" s="24" t="n">
         <v>272966</v>
       </c>
-      <c r="F24" s="23" t="n">
+      <c r="F24" s="24" t="n">
         <v>559966</v>
       </c>
     </row>
@@ -1587,7 +1590,7 @@
         </is>
       </c>
       <c r="B27" s="14" t="n">
-        <v>18200</v>
+        <v>-5300</v>
       </c>
       <c r="C27" s="14" t="n">
         <v>20900</v>
@@ -1596,7 +1599,7 @@
         <v>148400</v>
       </c>
       <c r="E27" s="14" t="n">
-        <v>-163900</v>
+        <v>-140400</v>
       </c>
       <c r="F27" s="13" t="inlineStr"/>
     </row>
@@ -1607,21 +1610,21 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>-5400</v>
+        <v>-28900</v>
       </c>
       <c r="C28" s="5" t="n">
-        <v>15500</v>
+        <v>-8000</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>163900</v>
-      </c>
-      <c r="E28" s="24" t="n">
+        <v>140400</v>
+      </c>
+      <c r="E28" s="25" t="n">
         <v>0</v>
       </c>
       <c r="F28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="25" t="inlineStr">
+      <c r="A29" s="26" t="inlineStr">
         <is>
           <t>⚠ Vigilar: el saldo se aprieta antes de la rifa (ago) y de los pagos grandes de sep (casa, transporte).</t>
         </is>
@@ -1651,7 +1654,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>OPTIMIZACIÓN · palancas para cerrar (o reducir) la brecha</t>
         </is>
@@ -1665,22 +1668,22 @@
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="27" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>Palanca</t>
         </is>
       </c>
-      <c r="B4" s="27" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>Impacto (RD$)</t>
         </is>
       </c>
-      <c r="C4" s="27" t="inlineStr">
+      <c r="C4" s="28" t="inlineStr">
         <is>
           <t>Cómo</t>
         </is>
       </c>
-      <c r="D4" s="27" t="inlineStr">
+      <c r="D4" s="28" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
@@ -1864,7 +1867,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="28" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>ESCENARIO DE CIERRE · UNA forma de cerrar la brecha — [ESCENARIO], a validar</t>
         </is>
@@ -1878,22 +1881,22 @@
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="29" t="inlineStr">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>Fuente variable</t>
         </is>
       </c>
-      <c r="B4" s="29" t="inlineStr">
+      <c r="B4" s="30" t="inlineStr">
         <is>
           <t>Monto (RD$)</t>
         </is>
       </c>
-      <c r="C4" s="29" t="inlineStr">
+      <c r="C4" s="30" t="inlineStr">
         <is>
           <t>Supuesto</t>
         </is>
       </c>
-      <c r="D4" s="29" t="inlineStr">
+      <c r="D4" s="30" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>

</xml_diff>